<commit_message>
Update dashboard title to TaxETS Dashboard
</commit_message>
<xml_diff>
--- a/docs/Domestic VAT Test.xlsx
+++ b/docs/Domestic VAT Test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Documents/UNDP 2023/New contract_TE for database/IT Consulting Firm/Database Design/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tax-ETS\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B06FDA-EEC8-0B4C-AEAF-DE74C3F063A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -235,8 +235,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="170" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -274,7 +274,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -284,13 +284,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -633,18 +633,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
-    <col min="6" max="7" width="12.5" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.5" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="7" width="12.42578125" customWidth="1"/>
+    <col min="9" max="9" width="16.85546875" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" customWidth="1"/>
+    <col min="11" max="11" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -679,7 +679,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -710,7 +710,7 @@
       </c>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -741,7 +741,7 @@
       </c>
       <c r="K3" s="6"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -772,7 +772,7 @@
       </c>
       <c r="K4" s="6"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -803,7 +803,7 @@
       </c>
       <c r="K5" s="6"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -834,7 +834,7 @@
       </c>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -865,7 +865,7 @@
       </c>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -896,7 +896,7 @@
       </c>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -927,7 +927,7 @@
       </c>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -958,7 +958,7 @@
       </c>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -989,7 +989,7 @@
       </c>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>1</v>
       </c>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>1</v>
       </c>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>1</v>
       </c>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>1</v>
       </c>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>1</v>
       </c>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>1</v>
       </c>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>1</v>
       </c>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>1</v>
       </c>

</xml_diff>